<commit_message>
file sent to menaka dd
</commit_message>
<xml_diff>
--- a/drg/menaka dd/archi/from menaka dd/3. slab design.xlsx
+++ b/drg/menaka dd/archi/from menaka dd/3. slab design.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\drg\menaka dd\excel for calculation\from menaka dd\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\drg\menaka dd\archi\from menaka dd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638F0988-1FD2-4636-BEED-0C6C36B1F7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217417ED-865D-4297-8F53-F57AFF2D0D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="5985" yWindow="750" windowWidth="13050" windowHeight="10050" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="two way slab design" sheetId="1" r:id="rId1"/>
@@ -781,9 +781,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -1276,7 +1276,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1385,19 +1385,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1426,7 +1426,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1442,11 +1442,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1469,13 +1469,82 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1494,77 +1563,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2101,57 +2101,57 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T85"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" style="38" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="38" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" style="38" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="38"/>
-    <col min="5" max="5" width="10.88671875" style="38" customWidth="1"/>
-    <col min="6" max="9" width="9.109375" style="38"/>
-    <col min="10" max="10" width="6.33203125" style="38" customWidth="1"/>
-    <col min="11" max="11" width="9.5546875" style="38" customWidth="1"/>
-    <col min="12" max="12" width="8.33203125" style="38" customWidth="1"/>
-    <col min="13" max="13" width="7.88671875" style="38" customWidth="1"/>
-    <col min="14" max="14" width="8.6640625" style="38" customWidth="1"/>
-    <col min="15" max="15" width="7.5546875" style="38" customWidth="1"/>
-    <col min="16" max="16384" width="9.109375" style="38"/>
+    <col min="1" max="1" width="28.5703125" style="38" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="38" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="38"/>
+    <col min="5" max="5" width="10.85546875" style="38" customWidth="1"/>
+    <col min="6" max="9" width="9.140625" style="38"/>
+    <col min="10" max="10" width="6.28515625" style="38" customWidth="1"/>
+    <col min="11" max="11" width="9.5703125" style="38" customWidth="1"/>
+    <col min="12" max="12" width="8.28515625" style="38" customWidth="1"/>
+    <col min="13" max="13" width="7.85546875" style="38" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" style="38" customWidth="1"/>
+    <col min="15" max="15" width="7.5703125" style="38" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
         <v>120</v>
       </c>
       <c r="D2" s="38">
         <f>'Input values and Results'!B3</f>
-        <v>4521.2</v>
+        <v>4800.5999999999995</v>
       </c>
       <c r="E2" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
         <v>121</v>
       </c>
       <c r="D3" s="38">
         <f>'Input values and Results'!B4</f>
-        <v>3454.3999999999996</v>
+        <v>4267.2</v>
       </c>
       <c r="E3" s="38" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="38">
         <f>D3*2</f>
-        <v>6908.7999999999993</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>8534.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>122</v>
       </c>
@@ -2162,60 +2162,60 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
         <v>124</v>
       </c>
       <c r="D5" s="38">
         <f>D2-D4</f>
-        <v>4291.2</v>
+        <v>4570.5999999999995</v>
       </c>
       <c r="E5" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>123</v>
       </c>
       <c r="D6" s="38">
         <f>D3-D4</f>
-        <v>3224.3999999999996</v>
+        <v>4037.2</v>
       </c>
       <c r="E6" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>126</v>
       </c>
       <c r="D7" s="38">
         <f>D5+0.5*D12</f>
-        <v>4343.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>4623.0999999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>125</v>
       </c>
       <c r="D8" s="38">
         <f>D6+0.5*D12</f>
-        <v>3276.8999999999996</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>4089.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>1</v>
       </c>
       <c r="D10" s="35">
         <f>MIN(D2,D7)</f>
-        <v>4343.7</v>
+        <v>4623.0999999999995</v>
       </c>
       <c r="E10" s="38" t="s">
         <v>13</v>
@@ -2224,13 +2224,13 @@
         <v>128</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
         <v>2</v>
       </c>
       <c r="D11" s="35">
         <f>MIN(D3,D8)</f>
-        <v>3276.8999999999996</v>
+        <v>4089.7</v>
       </c>
       <c r="E11" s="38" t="s">
         <v>13</v>
@@ -2240,10 +2240,10 @@
       </c>
       <c r="J11" s="38">
         <f>D11/1000</f>
-        <v>3.2768999999999995</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>4.0896999999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="38" t="s">
         <v>3</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
         <v>59</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="38" t="s">
         <v>60</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="38" t="s">
         <v>77</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
         <v>47</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
         <v>6</v>
       </c>
@@ -2314,22 +2314,22 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="D18" s="39"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B19" s="38" t="s">
         <v>40</v>
       </c>
       <c r="D19" s="40">
         <f>D10/D11</f>
-        <v>1.3255515883914677</v>
+        <v>1.1304252145634153</v>
       </c>
       <c r="E19" s="38" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="38" t="s">
         <v>11</v>
       </c>
@@ -2338,13 +2338,13 @@
         <v>&lt;2 two way slab</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A21" s="86" t="str">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21" s="94" t="str">
         <f>'Input values and Results'!A12</f>
-        <v>One Short Edge Discontinuous</v>
-      </c>
-      <c r="B21" s="86"/>
-      <c r="C21" s="86"/>
+        <v>Two Adjacent Edge Discontinuous</v>
+      </c>
+      <c r="B21" s="94"/>
+      <c r="C21" s="94"/>
       <c r="D21" s="39"/>
       <c r="E21" s="39"/>
       <c r="F21" s="39"/>
@@ -2354,10 +2354,10 @@
       <c r="L21" s="37"/>
       <c r="T21" s="38" t="str">
         <f>A21</f>
-        <v>One Short Edge Discontinuous</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+        <v>Two Adjacent Edge Discontinuous</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I22" s="73"/>
       <c r="J22" s="73" t="s">
         <v>244</v>
@@ -2367,7 +2367,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I23" s="74"/>
       <c r="J23" s="73" t="s">
         <v>240</v>
@@ -2377,7 +2377,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="38" t="s">
         <v>4</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="38" t="s">
         <v>5</v>
       </c>
@@ -2410,7 +2410,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="38" t="s">
         <v>7</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="38" t="s">
         <v>107</v>
       </c>
@@ -2440,7 +2440,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="38" t="s">
         <v>8</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C29" s="38" t="s">
         <v>64</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="38" t="s">
         <v>9</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C31" s="38" t="s">
         <v>236</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="38" t="s">
         <v>61</v>
       </c>
@@ -2502,21 +2502,21 @@
       </c>
       <c r="H32" s="41"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A33" s="85" t="s">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A33" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="85" t="s">
+      <c r="B33" s="93" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="84" t="s">
+      <c r="C33" s="92" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="84"/>
-      <c r="E33" s="84" t="s">
+      <c r="D33" s="92"/>
+      <c r="E33" s="92" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="84"/>
+      <c r="F33" s="92"/>
       <c r="J33" s="50"/>
       <c r="K33" s="50"/>
       <c r="L33" s="51"/>
@@ -2524,9 +2524,9 @@
       <c r="N33" s="51"/>
       <c r="O33" s="51"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A34" s="85"/>
-      <c r="B34" s="85"/>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A34" s="93"/>
+      <c r="B34" s="93"/>
       <c r="C34" s="37" t="s">
         <v>19</v>
       </c>
@@ -2542,7 +2542,7 @@
       <c r="J34" s="50"/>
       <c r="K34" s="50"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="37">
         <v>1</v>
       </c>
@@ -2551,26 +2551,26 @@
       </c>
       <c r="C35" s="37">
         <f>'alpha value'!L8</f>
-        <v>5.2022063535658705E-2</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="D35" s="37">
         <f>'alpha value'!L9</f>
-        <v>3.9511031767829351E-2</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="E35" s="37">
         <f>'alpha value'!M8</f>
-        <v>3.6999999999999998E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="F35" s="37">
         <f>'alpha value'!M9</f>
-        <v>2.8000000000000001E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="L35" s="41"/>
       <c r="M35" s="41"/>
       <c r="N35" s="41"/>
       <c r="O35" s="41"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="37">
         <v>2</v>
       </c>
@@ -2579,26 +2579,26 @@
       </c>
       <c r="C36" s="37">
         <f>C35*$D$30*$D$11*$D$11/10^6</f>
-        <v>6.5986603309068741</v>
+        <v>10.892081088866247</v>
       </c>
       <c r="D36" s="37">
         <f>D35*$D$30*$D$11*$D$11/10^6</f>
-        <v>5.011717341448124</v>
+        <v>8.2034258372718725</v>
       </c>
       <c r="E36" s="37">
         <f>E35*$D$30*$D$11*$D$11/10^6</f>
-        <v>4.6932092971706236</v>
+        <v>9.2858696385918762</v>
       </c>
       <c r="F36" s="37">
         <f>F35*$D$30*$D$11*$D$11/10^6</f>
-        <v>3.551617846507499</v>
+        <v>6.9150093053343742</v>
       </c>
       <c r="L36" s="41"/>
       <c r="M36" s="41"/>
       <c r="N36" s="41"/>
       <c r="O36" s="41"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="37">
         <v>3</v>
       </c>
@@ -2607,26 +2607,26 @@
       </c>
       <c r="C37" s="37">
         <f>'steel area calculation'!L7</f>
-        <v>149.81242025653103</v>
+        <v>253.80294639829856</v>
       </c>
       <c r="D37" s="37">
         <f>'steel area calculation'!L8</f>
-        <v>112.75184290675337</v>
+        <v>188.01940270931087</v>
       </c>
       <c r="E37" s="37">
         <f>'steel area calculation'!L9</f>
-        <v>105.39653582479998</v>
+        <v>214.22772530757535</v>
       </c>
       <c r="F37" s="37">
         <f>'steel area calculation'!L10</f>
-        <v>79.253643083059629</v>
+        <v>157.28475003624399</v>
       </c>
       <c r="L37" s="49"/>
       <c r="M37" s="49"/>
       <c r="N37" s="49"/>
       <c r="O37" s="49"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="37">
         <v>4</v>
       </c>
@@ -2650,33 +2650,33 @@
         <v>150</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="37"/>
       <c r="B39" s="37" t="s">
         <v>62</v>
       </c>
       <c r="C39" s="37">
         <f>IF(C37&gt;C38,C37,C38)</f>
-        <v>150</v>
+        <v>253.80294639829856</v>
       </c>
       <c r="D39" s="37">
         <f t="shared" ref="D39:F39" si="1">IF(D37&gt;D38,D37,D38)</f>
-        <v>150</v>
+        <v>188.01940270931087</v>
       </c>
       <c r="E39" s="37">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>214.22772530757535</v>
       </c>
       <c r="F39" s="37">
         <f t="shared" si="1"/>
-        <v>150</v>
+        <v>157.28475003624399</v>
       </c>
       <c r="L39" s="41"/>
       <c r="M39" s="41"/>
       <c r="N39" s="41"/>
       <c r="O39" s="41"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="37">
         <v>5</v>
       </c>
@@ -2685,26 +2685,26 @@
       </c>
       <c r="C40" s="37">
         <f>1000/(C39/(22*$C$32*$C$32/(4*7)))</f>
-        <v>523.80952380952374</v>
+        <v>309.57650289892496</v>
       </c>
       <c r="D40" s="37">
         <f>1000/(D39/(22*$C$32*$C$32/(4*7)))</f>
-        <v>523.80952380952374</v>
+        <v>417.89000198508586</v>
       </c>
       <c r="E40" s="37">
         <f t="shared" ref="E40:F40" si="2">1000/(E39/(22*$D$32*$D$32/(4*7)))</f>
-        <v>335.23809523809524</v>
+        <v>234.73018823085135</v>
       </c>
       <c r="F40" s="37">
         <f t="shared" si="2"/>
-        <v>335.23809523809524</v>
+        <v>319.7113151410208</v>
       </c>
       <c r="L40" s="49"/>
       <c r="M40" s="49"/>
       <c r="N40" s="49"/>
       <c r="O40" s="49"/>
     </row>
-    <row r="41" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="37"/>
       <c r="B41" s="37"/>
       <c r="C41" s="37">
@@ -2720,7 +2720,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="37"/>
       <c r="B42" s="37" t="s">
         <v>63</v>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="E42" s="37">
         <f t="shared" si="3"/>
-        <v>300</v>
+        <v>234.73018823085135</v>
       </c>
       <c r="F42" s="37">
         <f t="shared" si="3"/>
@@ -2746,7 +2746,7 @@
         <v>0.2681904761904762</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="37">
         <v>6</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="37">
         <v>7</v>
       </c>
@@ -2798,7 +2798,7 @@
       <c r="N44" s="49"/>
       <c r="O44" s="49"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="38">
         <v>8</v>
       </c>
@@ -2822,27 +2822,27 @@
         <v>0.2681904761904762</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A46" s="83" t="s">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" s="97" t="s">
         <v>65</v>
       </c>
-      <c r="B46" s="83"/>
-      <c r="C46" s="83"/>
-      <c r="D46" s="83"/>
-      <c r="E46" s="83"/>
-      <c r="F46" s="83"/>
-      <c r="G46" s="83"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B46" s="97"/>
+      <c r="C46" s="97"/>
+      <c r="D46" s="97"/>
+      <c r="E46" s="97"/>
+      <c r="F46" s="97"/>
+      <c r="G46" s="97"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="38" t="s">
         <v>66</v>
       </c>
       <c r="D47" s="38">
         <f>D11</f>
-        <v>3276.8999999999996</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
+        <v>4089.7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="38" t="s">
         <v>67</v>
       </c>
@@ -2851,16 +2851,16 @@
         <v>105</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="38" t="s">
         <v>68</v>
       </c>
       <c r="D49" s="41">
         <f>D47/D48</f>
-        <v>31.208571428571425</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+        <v>38.949523809523811</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="38" t="s">
         <v>69</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="38" t="s">
         <v>70</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="38" t="s">
         <v>72</v>
       </c>
@@ -2890,19 +2890,19 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="38" t="s">
         <v>76</v>
       </c>
       <c r="D53" s="43">
         <f>0.58*D15*D39/D44</f>
-        <v>83.045454545454533</v>
+        <v>104.09437840906392</v>
       </c>
       <c r="E53" s="38" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="38" t="s">
         <v>79</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>0.41904761904761906</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="38" t="s">
         <v>73</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="38" t="s">
         <v>205</v>
       </c>
@@ -2935,36 +2935,36 @@
         <v>OK Safe</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A59" s="83" t="s">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B59" s="83"/>
-      <c r="C59" s="83"/>
-      <c r="D59" s="83"/>
-      <c r="E59" s="83"/>
-      <c r="F59" s="83"/>
-      <c r="G59" s="83"/>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B59" s="97"/>
+      <c r="C59" s="97"/>
+      <c r="D59" s="97"/>
+      <c r="E59" s="97"/>
+      <c r="F59" s="97"/>
+      <c r="G59" s="97"/>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="38" t="s">
         <v>81</v>
       </c>
       <c r="D60" s="44">
         <f>D30*D11/2000</f>
-        <v>19.354190624999998</v>
+        <v>24.154790624999997</v>
       </c>
       <c r="E60" s="38" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="38" t="s">
         <v>83</v>
       </c>
       <c r="D61" s="41">
         <f>D60/(1000*D48)*1000</f>
-        <v>0.18432562499999997</v>
+        <v>0.23004562499999998</v>
       </c>
       <c r="E61" s="38" t="s">
         <v>78</v>
@@ -2973,7 +2973,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="38" t="s">
         <v>85</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="38" t="s">
         <v>47</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="38" t="s">
         <v>84</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>OK Safe</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="38" t="s">
         <v>100</v>
       </c>
@@ -3051,12 +3051,12 @@
         <v>125</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="38" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="38" t="s">
         <v>87</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>0.24943310657596371</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="38" t="s">
         <v>88</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="38" t="s">
         <v>90</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="38" t="s">
         <v>104</v>
       </c>
@@ -3102,55 +3102,55 @@
         <v>OK Safe</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="38" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B75" s="38" t="s">
         <v>130</v>
       </c>
       <c r="C75" s="38">
         <f>D11*0.2</f>
-        <v>655.38</v>
+        <v>817.94</v>
       </c>
       <c r="D75" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B76" s="38" t="s">
         <v>131</v>
       </c>
       <c r="C76" s="38">
         <f>C75*C75</f>
-        <v>429522.94439999998</v>
+        <v>669025.84360000014</v>
       </c>
       <c r="D76" s="38" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="81" t="s">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="95" t="s">
         <v>109</v>
       </c>
-      <c r="B77" s="81"/>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="82" t="s">
+      <c r="B77" s="95"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="96" t="s">
         <v>110</v>
       </c>
-      <c r="B78" s="82"/>
-      <c r="C78" s="82"/>
-      <c r="D78" s="82"/>
-      <c r="E78" s="82"/>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="81" t="s">
+      <c r="B78" s="96"/>
+      <c r="C78" s="96"/>
+      <c r="D78" s="96"/>
+      <c r="E78" s="96"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="95" t="s">
         <v>111</v>
       </c>
-      <c r="B79" s="81"/>
+      <c r="B79" s="95"/>
       <c r="D79" s="46">
         <v>0.375</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C80" s="38" t="s">
         <v>114</v>
       </c>
@@ -3170,25 +3170,25 @@
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C81" s="38" t="s">
         <v>116</v>
       </c>
       <c r="D81" s="38">
         <f>0.2*D11</f>
-        <v>655.38</v>
+        <v>817.94</v>
       </c>
       <c r="E81" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="81" t="s">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="95" t="s">
         <v>117</v>
       </c>
-      <c r="B82" s="81"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B82" s="95"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C83" s="38" t="s">
         <v>112</v>
       </c>
@@ -3199,19 +3199,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C84" s="38" t="s">
         <v>118</v>
       </c>
       <c r="D84" s="38">
         <f>D81/(D80)*(22*D83^2/(4*7))</f>
-        <v>167.77727999999999</v>
+        <v>209.39264</v>
       </c>
       <c r="E84" s="38" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C85" s="38" t="s">
         <v>119</v>
       </c>
@@ -3224,17 +3224,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A77:B77"/>
     <mergeCell ref="A82:B82"/>
     <mergeCell ref="A78:E78"/>
     <mergeCell ref="A79:B79"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="A59:G59"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A21:C21"/>
   </mergeCells>
   <conditionalFormatting sqref="F56">
     <cfRule type="cellIs" dxfId="9" priority="8" operator="equal">
@@ -3283,50 +3283,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H134"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.33203125" style="52" customWidth="1"/>
-    <col min="2" max="2" width="39.44140625" style="52" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" style="52" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" style="52" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" style="52" customWidth="1"/>
+    <col min="2" max="2" width="39.42578125" style="52" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="52" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" style="52" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="52" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" style="52" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="52"/>
+    <col min="6" max="6" width="8.140625" style="52" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="52"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="76" t="s">
+    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="99" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="77" t="s">
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="77"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="100"/>
+      <c r="C2" s="100"/>
+      <c r="D2" s="100"/>
+      <c r="E2" s="100"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="53"/>
       <c r="B3" s="53"/>
       <c r="C3" s="53"/>
       <c r="D3" s="53"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="53"/>
       <c r="B4" s="53"/>
       <c r="C4" s="53"/>
       <c r="D4" s="53"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="6" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" s="54" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="54">
         <v>1</v>
       </c>
@@ -3334,36 +3334,36 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" s="52" t="s">
         <v>150</v>
       </c>
       <c r="C7" s="72">
         <f>'two way slab design'!D2/1000</f>
-        <v>4.5211999999999994</v>
+        <v>4.8005999999999993</v>
       </c>
       <c r="D7" s="52" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" s="52" t="s">
         <v>151</v>
       </c>
       <c r="C8" s="72">
         <f>'two way slab design'!D3/1000</f>
-        <v>3.4543999999999997</v>
+        <v>4.2671999999999999</v>
       </c>
       <c r="D8" s="52" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10" s="52" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" s="52" t="s">
         <v>145</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" s="52" t="s">
         <v>146</v>
       </c>
@@ -3393,10 +3393,10 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="54"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="54">
         <v>2</v>
       </c>
@@ -3404,14 +3404,14 @@
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="54"/>
       <c r="B16" s="52" t="s">
         <v>150</v>
       </c>
       <c r="C16" s="55">
         <f>'two way slab design'!D10/1000</f>
-        <v>4.3437000000000001</v>
+        <v>4.6230999999999991</v>
       </c>
       <c r="D16" s="52" t="s">
         <v>143</v>
@@ -3421,30 +3421,30 @@
         <v>1.0526315789473684</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="54"/>
       <c r="B17" s="52" t="s">
         <v>151</v>
       </c>
       <c r="C17" s="55">
         <f>'two way slab design'!D11/1000</f>
-        <v>3.2768999999999995</v>
+        <v>4.0896999999999997</v>
       </c>
       <c r="D17" s="52" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="54"/>
       <c r="B18" s="47" t="s">
         <v>40</v>
       </c>
       <c r="C18" s="55">
         <f>'two way slab design'!D19</f>
-        <v>1.3255515883914677</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1.1304252145634153</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="54"/>
       <c r="B19" s="47" t="s">
         <v>11</v>
@@ -3454,32 +3454,32 @@
         <v>&lt;2 two way slab</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="54"/>
       <c r="B20" s="47" t="s">
         <v>174</v>
       </c>
       <c r="C20" s="47"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="54"/>
       <c r="B21" s="57" t="str">
         <f>'Input values and Results'!A12</f>
-        <v>One Short Edge Discontinuous</v>
+        <v>Two Adjacent Edge Discontinuous</v>
       </c>
       <c r="C21" s="58"/>
       <c r="D21" s="58"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="54"/>
       <c r="B22" s="57"/>
       <c r="C22" s="58"/>
       <c r="D22" s="58"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="54"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="54">
         <v>3</v>
       </c>
@@ -3487,12 +3487,12 @@
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B25" s="54" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="59" t="s">
         <v>154</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B27" s="52" t="s">
         <v>156</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B28" s="52" t="s">
         <v>157</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="59" t="s">
         <v>158</v>
       </c>
@@ -3545,7 +3545,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B30" s="52" t="s">
         <v>160</v>
       </c>
@@ -3556,7 +3556,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B31" s="52" t="s">
         <v>161</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="59" t="s">
         <v>162</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B33" s="52" t="s">
         <v>164</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" s="52" t="s">
         <v>165</v>
       </c>
@@ -3605,7 +3605,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="59" t="s">
         <v>166</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B36" s="52" t="s">
         <v>168</v>
       </c>
@@ -3630,7 +3630,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B37" s="52" t="s">
         <v>169</v>
       </c>
@@ -3642,7 +3642,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B38" s="54" t="s">
         <v>170</v>
       </c>
@@ -3654,12 +3654,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B40" s="54" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B41" s="52" t="s">
         <v>235</v>
       </c>
@@ -3671,7 +3671,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B43" s="54" t="s">
         <v>172</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B44" s="52" t="s">
         <v>173</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="54">
         <v>4</v>
       </c>
@@ -3703,20 +3703,20 @@
         <v>175</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B47" s="52" t="s">
         <v>176</v>
       </c>
-      <c r="C47" s="78" t="s">
+      <c r="C47" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="D47" s="78"/>
-      <c r="E47" s="78" t="s">
+      <c r="D47" s="101"/>
+      <c r="E47" s="101" t="s">
         <v>18</v>
       </c>
-      <c r="F47" s="78"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F47" s="101"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B48" s="52" t="s">
         <v>181</v>
       </c>
@@ -3725,17 +3725,17 @@
       </c>
       <c r="D48" s="61">
         <f>'two way slab design'!C35</f>
-        <v>5.2022063535658705E-2</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="E48" s="60" t="s">
         <v>178</v>
       </c>
       <c r="F48" s="62">
         <f>'two way slab design'!E35</f>
-        <v>3.6999999999999998E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4.7E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B49" s="52" t="s">
         <v>182</v>
       </c>
@@ -3744,78 +3744,78 @@
       </c>
       <c r="D49" s="63">
         <f>'two way slab design'!D35</f>
-        <v>3.9511031767829351E-2</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="E49" s="60" t="s">
         <v>179</v>
       </c>
       <c r="F49" s="62">
         <f>'two way slab design'!F35</f>
-        <v>2.8000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B50" s="52" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B51" s="52" t="s">
         <v>183</v>
       </c>
       <c r="C51" s="55">
         <f>'two way slab design'!C36</f>
-        <v>6.5986603309068741</v>
+        <v>10.892081088866247</v>
       </c>
       <c r="D51" s="52" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B52" s="52" t="s">
         <v>184</v>
       </c>
       <c r="C52" s="55">
         <f>'two way slab design'!E36</f>
-        <v>4.6932092971706236</v>
+        <v>9.2858696385918762</v>
       </c>
       <c r="D52" s="52" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B53" s="52" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B54" s="52" t="s">
         <v>186</v>
       </c>
       <c r="C54" s="55">
         <f>'two way slab design'!D36</f>
-        <v>5.011717341448124</v>
+        <v>8.2034258372718725</v>
       </c>
       <c r="D54" s="52" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B55" s="52" t="s">
         <v>187</v>
       </c>
       <c r="C55" s="55">
         <f>'two way slab design'!F36</f>
-        <v>3.551617846507499</v>
+        <v>6.9150093053343742</v>
       </c>
       <c r="D55" s="52" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C56" s="55"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="54">
         <v>5</v>
       </c>
@@ -3823,31 +3823,31 @@
         <v>189</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B58" s="52" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B59" s="52" t="s">
         <v>191</v>
       </c>
       <c r="C59" s="55">
         <f>MAX(C51,C52,C54,C55)</f>
-        <v>6.5986603309068741</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10.892081088866247</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B60" s="52" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B61" s="52" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B63" s="52" t="s">
         <v>231</v>
       </c>
@@ -3855,7 +3855,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B64" s="52" t="s">
         <v>194</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B65" s="52" t="s">
         <v>195</v>
       </c>
@@ -3878,7 +3878,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="54">
         <v>6</v>
       </c>
@@ -3894,11 +3894,11 @@
         <v>Dist. Bar</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="80" t="s">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="103" t="s">
         <v>61</v>
       </c>
-      <c r="B68" s="80"/>
+      <c r="B68" s="103"/>
       <c r="C68" s="64">
         <f>'two way slab design'!C32</f>
         <v>10</v>
@@ -3912,25 +3912,25 @@
       </c>
       <c r="F68" s="47"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="79" t="s">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="102" t="s">
         <v>15</v>
       </c>
-      <c r="B69" s="79" t="s">
+      <c r="B69" s="102" t="s">
         <v>16</v>
       </c>
-      <c r="C69" s="78" t="s">
+      <c r="C69" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="D69" s="78"/>
-      <c r="E69" s="78" t="s">
+      <c r="D69" s="101"/>
+      <c r="E69" s="101" t="s">
         <v>18</v>
       </c>
-      <c r="F69" s="78"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="79"/>
-      <c r="B70" s="79"/>
+      <c r="F69" s="101"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="102"/>
+      <c r="B70" s="102"/>
       <c r="C70" s="60" t="s">
         <v>19</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="60">
         <v>1</v>
       </c>
@@ -3953,22 +3953,22 @@
       </c>
       <c r="C71" s="61">
         <f>'two way slab design'!C35</f>
-        <v>5.2022063535658705E-2</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="D71" s="61">
         <f>'two way slab design'!D35</f>
-        <v>3.9511031767829351E-2</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="E71" s="61">
         <f>'two way slab design'!E35</f>
-        <v>3.6999999999999998E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="F71" s="61">
         <f>'two way slab design'!F35</f>
-        <v>2.8000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+        <v>3.5000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="60">
         <v>2</v>
       </c>
@@ -3977,22 +3977,22 @@
       </c>
       <c r="C72" s="65">
         <f>'two way slab design'!C36</f>
-        <v>6.5986603309068741</v>
+        <v>10.892081088866247</v>
       </c>
       <c r="D72" s="65">
         <f>'two way slab design'!D36</f>
-        <v>5.011717341448124</v>
+        <v>8.2034258372718725</v>
       </c>
       <c r="E72" s="65">
         <f>'two way slab design'!E36</f>
-        <v>4.6932092971706236</v>
+        <v>9.2858696385918762</v>
       </c>
       <c r="F72" s="65">
         <f>'two way slab design'!F36</f>
-        <v>3.551617846507499</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+        <v>6.9150093053343742</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="60">
         <v>3</v>
       </c>
@@ -4001,22 +4001,22 @@
       </c>
       <c r="C73" s="65">
         <f>'two way slab design'!C37</f>
-        <v>149.81242025653103</v>
+        <v>253.80294639829856</v>
       </c>
       <c r="D73" s="65">
         <f>'two way slab design'!D37</f>
-        <v>112.75184290675337</v>
+        <v>188.01940270931087</v>
       </c>
       <c r="E73" s="65">
         <f>'two way slab design'!E37</f>
-        <v>105.39653582479998</v>
+        <v>214.22772530757535</v>
       </c>
       <c r="F73" s="65">
         <f>'two way slab design'!F37</f>
-        <v>79.253643083059629</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+        <v>157.28475003624399</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="60">
         <v>4</v>
       </c>
@@ -4040,29 +4040,29 @@
         <v>150</v>
       </c>
     </row>
-    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="60"/>
       <c r="B75" s="60" t="s">
         <v>62</v>
       </c>
       <c r="C75" s="65">
         <f>'two way slab design'!C39</f>
-        <v>150</v>
+        <v>253.80294639829856</v>
       </c>
       <c r="D75" s="65">
         <f>'two way slab design'!D39</f>
-        <v>150</v>
+        <v>188.01940270931087</v>
       </c>
       <c r="E75" s="65">
         <f>'two way slab design'!E39</f>
-        <v>150</v>
+        <v>214.22772530757535</v>
       </c>
       <c r="F75" s="65">
         <f>'two way slab design'!F39</f>
-        <v>150</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+        <v>157.28475003624399</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="60">
         <v>5</v>
       </c>
@@ -4071,22 +4071,22 @@
       </c>
       <c r="C76" s="65">
         <f>'two way slab design'!C40</f>
-        <v>523.80952380952374</v>
+        <v>309.57650289892496</v>
       </c>
       <c r="D76" s="65">
         <f>'two way slab design'!D40</f>
-        <v>523.80952380952374</v>
+        <v>417.89000198508586</v>
       </c>
       <c r="E76" s="65">
         <f>'two way slab design'!E40</f>
-        <v>335.23809523809524</v>
+        <v>234.73018823085135</v>
       </c>
       <c r="F76" s="65">
         <f>'two way slab design'!F40</f>
-        <v>335.23809523809524</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+        <v>319.7113151410208</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="60"/>
       <c r="B77" s="60"/>
       <c r="C77" s="65">
@@ -4106,7 +4106,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="60"/>
       <c r="B78" s="60" t="s">
         <v>63</v>
@@ -4121,14 +4121,14 @@
       </c>
       <c r="E78" s="65">
         <f>'two way slab design'!E42</f>
-        <v>300</v>
+        <v>234.73018823085135</v>
       </c>
       <c r="F78" s="65">
         <f>'two way slab design'!F42</f>
         <v>300</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="60">
         <v>6</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="60">
         <v>7</v>
       </c>
@@ -4176,7 +4176,7 @@
         <v>335.23809523809524</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="60">
         <v>8</v>
       </c>
@@ -4200,7 +4200,7 @@
         <v>0.2681904761904762</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="47"/>
       <c r="B82" s="47"/>
       <c r="C82" s="66"/>
@@ -4208,7 +4208,7 @@
       <c r="E82" s="66"/>
       <c r="F82" s="66"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="54">
         <v>7</v>
       </c>
@@ -4216,7 +4216,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="67">
         <v>7.1</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="47" t="s">
         <v>199</v>
       </c>
@@ -4235,17 +4235,17 @@
       <c r="D85" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="E85" s="75" t="s">
+      <c r="E85" s="98" t="s">
         <v>200</v>
       </c>
-      <c r="F85" s="75"/>
-      <c r="G85" s="75"/>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F85" s="98"/>
+      <c r="G85" s="98"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E86" s="68"/>
       <c r="F86" s="68"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="54">
         <v>7.2</v>
       </c>
@@ -4253,12 +4253,12 @@
         <v>201</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B88" s="47" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B89" s="47" t="s">
         <v>206</v>
       </c>
@@ -4266,16 +4266,16 @@
         <v>203</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B90" s="47" t="s">
         <v>68</v>
       </c>
       <c r="C90" s="52">
         <f>'two way slab design'!D49</f>
-        <v>31.208571428571425</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+        <v>38.949523809523811</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B91" s="56" t="s">
         <v>204</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B92" s="69" t="s">
         <v>233</v>
       </c>
@@ -4295,7 +4295,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B93" s="69" t="s">
         <v>234</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B94" s="59" t="s">
         <v>207</v>
       </c>
@@ -4321,24 +4321,24 @@
         <v>213</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B95" s="52" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="52" t="s">
         <v>212</v>
       </c>
       <c r="C96" s="55">
         <f>'two way slab design'!D53</f>
-        <v>83.045454545454533</v>
+        <v>104.09437840906392</v>
       </c>
       <c r="D96" s="52" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B97" s="47" t="s">
         <v>79</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>0.41904761904761906</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B98" s="47" t="s">
         <v>73</v>
       </c>
@@ -4356,7 +4356,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B99" s="47" t="s">
         <v>205</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>OK Safe</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B100" s="47" t="s">
         <v>214</v>
       </c>
@@ -4378,7 +4378,7 @@
         <v>SAFE</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="54">
         <v>7.3</v>
       </c>
@@ -4386,36 +4386,36 @@
         <v>215</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B103" s="47" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B104" s="47" t="s">
         <v>217</v>
       </c>
       <c r="C104" s="55">
         <f>'two way slab design'!D60</f>
-        <v>19.354190624999998</v>
+        <v>24.154790624999997</v>
       </c>
       <c r="D104" s="52" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B105" s="47" t="s">
         <v>218</v>
       </c>
       <c r="C105" s="55">
         <f>'two way slab design'!D61</f>
-        <v>0.18432562499999997</v>
+        <v>0.23004562499999998</v>
       </c>
       <c r="D105" s="52" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B106" s="47" t="s">
         <v>220</v>
       </c>
@@ -4424,19 +4424,19 @@
         <v>0.24943310657596371</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B107" s="47" t="s">
         <v>221</v>
       </c>
       <c r="C107" s="55"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B108" s="47" t="s">
         <v>222</v>
       </c>
       <c r="C108" s="55"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B109" s="59" t="s">
         <v>88</v>
       </c>
@@ -4448,12 +4448,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B110" s="47" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B111" s="70" t="s">
         <v>229</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B112" s="59" t="s">
         <v>223</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B113" s="59" t="s">
         <v>224</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>OK Safe</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="54">
         <v>8</v>
       </c>
@@ -4491,7 +4491,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B116" s="59" t="s">
         <v>226</v>
       </c>
@@ -4503,7 +4503,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B117" s="59" t="s">
         <v>227</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>10mm ø @ 150mm c/c</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B118" s="59" t="s">
         <v>228</v>
       </c>
@@ -4521,7 +4521,7 @@
         <v>10mm ø @ 150mm c/c</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B119" s="59" t="s">
         <v>238</v>
       </c>
@@ -4530,7 +4530,7 @@
         <v>8mm ø @ 150mm c/c</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B120" s="59" t="s">
         <v>239</v>
       </c>
@@ -4539,10 +4539,10 @@
         <v>8mm ø @ 150mm c/c</v>
       </c>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="59"/>
     </row>
-    <row r="134" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="134" spans="2:2" ht="20.25" x14ac:dyDescent="0.3">
       <c r="B134" s="71"/>
     </row>
   </sheetData>
@@ -4566,17 +4566,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:S42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>87</v>
       </c>
@@ -4584,14 +4584,14 @@
         <f>'two way slab design'!D68</f>
         <v>0.24943310657596371</v>
       </c>
-      <c r="G2" s="87" t="s">
+      <c r="G2" s="104" t="s">
         <v>98</v>
       </c>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
-      <c r="J2" s="87"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="104"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -4600,7 +4600,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>97</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>0.35954648526077093</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G5" t="s">
         <v>94</v>
       </c>
@@ -4617,7 +4617,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>87</v>
       </c>
@@ -4640,7 +4640,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="28">
         <v>0</v>
       </c>
@@ -4663,7 +4663,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f>IF(AND($C$2&gt;=A7,$C$2&lt;=A9),$C$2,0)</f>
         <v>0</v>
@@ -4697,7 +4697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28">
         <v>0.15</v>
       </c>
@@ -4720,7 +4720,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f>IF(AND($C$2&gt;=A9,$C$2&lt;=A11),$C$2,0)</f>
         <v>0.24943310657596371</v>
@@ -4754,7 +4754,7 @@
         <v>0.35954648526077093</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="28">
         <v>0.25</v>
       </c>
@@ -4777,7 +4777,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f>IF(AND($C$2&gt;=A11,$C$2&lt;=A13),$C$2,0)</f>
         <v>0</v>
@@ -4811,7 +4811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="28">
         <v>0.5</v>
       </c>
@@ -4834,7 +4834,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f>IF(AND($C$2&gt;=A13,$C$2&lt;=A15),$C$2,0)</f>
         <v>0</v>
@@ -4868,7 +4868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28">
         <v>0.75</v>
       </c>
@@ -4891,7 +4891,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f>IF(AND($C$2&gt;=A15,$C$2&lt;=A17),$C$2,0)</f>
         <v>0</v>
@@ -4925,7 +4925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="28">
         <v>1</v>
       </c>
@@ -4948,7 +4948,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <f>IF(AND($C$2&gt;=A17,$C$2&lt;=A19),$C$2,0)</f>
         <v>0</v>
@@ -4982,7 +4982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="28">
         <v>1.25</v>
       </c>
@@ -5005,7 +5005,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <f>IF(AND($C$2&gt;=A19,$C$2&lt;=A21),$C$2,0)</f>
         <v>0</v>
@@ -5039,7 +5039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="28">
         <v>1.5</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <f>IF(AND($C$2&gt;=A21,$C$2&lt;=A23),$C$2,0)</f>
         <v>0</v>
@@ -5096,7 +5096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="28">
         <v>1.75</v>
       </c>
@@ -5119,7 +5119,7 @@
         <v>0.84</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <f>IF(AND($C$2&gt;=A23,$C$2&lt;=A25),$C$2,0)</f>
         <v>0</v>
@@ -5153,7 +5153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="28">
         <v>2</v>
       </c>
@@ -5176,7 +5176,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
         <f>IF(AND($C$2&gt;=A25,$C$2&lt;=A27),$C$2,0)</f>
         <v>0</v>
@@ -5210,7 +5210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="28">
         <v>2.25</v>
       </c>
@@ -5233,7 +5233,7 @@
         <v>0.92</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
         <f>IF(AND($C$2&gt;=A27,$C$2&lt;=A29),$C$2,0)</f>
         <v>0</v>
@@ -5267,7 +5267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="28">
         <v>2.5</v>
       </c>
@@ -5290,7 +5290,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
         <f>IF(AND($C$2&gt;=A29,$C$2&lt;=A31),$C$2,0)</f>
         <v>0</v>
@@ -5324,7 +5324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="28">
         <v>2.75</v>
       </c>
@@ -5347,7 +5347,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <f>IF(AND($C$2&gt;=A31,$C$2&lt;=A33),$C$2,0)</f>
         <v>0</v>
@@ -5381,7 +5381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:19" s="28" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="28">
         <v>3</v>
       </c>
@@ -5404,13 +5404,13 @@
         <v>1.01</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="I34">
         <f>MAX(I8:I32)</f>
         <v>0.35954648526077093</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>101</v>
       </c>
@@ -5418,7 +5418,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
         <v>91</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>89</v>
       </c>
@@ -5484,7 +5484,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>90</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="C40">
         <f>C39</f>
         <v>0</v>
@@ -5580,7 +5580,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>102</v>
       </c>
@@ -5600,65 +5600,65 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A2:R18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B2">
         <f>(G2*12+H2)*25.4</f>
-        <v>3454.3999999999996</v>
+        <v>4800.5999999999995</v>
       </c>
       <c r="C2">
         <f>(I2*12+J2)*25.4</f>
-        <v>4521.2</v>
+        <v>4267.2</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="G2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I2">
         <v>14</v>
       </c>
       <c r="J2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3">
         <f>IF(B2&gt;C2,B2,C2)</f>
-        <v>4521.2</v>
+        <v>4800.5999999999995</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
         <f>IF(B2&lt;C2,B2,C2)</f>
-        <v>3454.3999999999996</v>
+        <v>4267.2</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -5680,7 +5680,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -5703,7 +5703,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -5714,7 +5714,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -5725,7 +5725,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="34" t="s">
         <v>106</v>
       </c>
@@ -5736,9 +5736,9 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
@@ -5747,7 +5747,7 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
@@ -5755,7 +5755,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
@@ -5763,7 +5763,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
@@ -5771,7 +5771,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="M16" s="33"/>
       <c r="N16" s="33"/>
       <c r="O16" s="33"/>
@@ -5779,7 +5779,7 @@
       <c r="Q16" s="33"/>
       <c r="R16" s="33"/>
     </row>
-    <row r="17" spans="13:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="13:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="M17" s="33"/>
       <c r="N17" s="33"/>
       <c r="O17" s="33"/>
@@ -5787,7 +5787,7 @@
       <c r="Q17" s="33"/>
       <c r="R17" s="33"/>
     </row>
-    <row r="18" spans="13:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="13:18" x14ac:dyDescent="0.25">
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
@@ -5816,46 +5816,46 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AB42"/>
-  <sheetFormatPr defaultColWidth="6.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="6.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" style="2"/>
-    <col min="2" max="2" width="6.6640625" style="4"/>
-    <col min="3" max="3" width="6.6640625" style="15"/>
-    <col min="4" max="4" width="6.6640625" style="4"/>
-    <col min="5" max="5" width="6.6640625" style="15"/>
-    <col min="6" max="6" width="6.6640625" style="4"/>
-    <col min="7" max="7" width="6.6640625" style="15"/>
-    <col min="8" max="8" width="6.6640625" style="4"/>
-    <col min="9" max="9" width="6.6640625" style="15"/>
-    <col min="10" max="10" width="6.6640625" style="4"/>
-    <col min="11" max="11" width="6.6640625" style="15"/>
-    <col min="12" max="12" width="6.6640625" style="4"/>
-    <col min="13" max="13" width="6.6640625" style="15"/>
-    <col min="14" max="14" width="6.6640625" style="4"/>
-    <col min="15" max="15" width="6.6640625" style="15"/>
-    <col min="16" max="16" width="8.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.6640625" style="15"/>
-    <col min="18" max="18" width="6.6640625" style="26"/>
-    <col min="19" max="22" width="6.6640625" style="4"/>
-    <col min="23" max="23" width="30.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="6.6640625" style="4"/>
+    <col min="1" max="1" width="6.7109375" style="2"/>
+    <col min="2" max="2" width="6.7109375" style="4"/>
+    <col min="3" max="3" width="6.7109375" style="15"/>
+    <col min="4" max="4" width="6.7109375" style="4"/>
+    <col min="5" max="5" width="6.7109375" style="15"/>
+    <col min="6" max="6" width="6.7109375" style="4"/>
+    <col min="7" max="7" width="6.7109375" style="15"/>
+    <col min="8" max="8" width="6.7109375" style="4"/>
+    <col min="9" max="9" width="6.7109375" style="15"/>
+    <col min="10" max="10" width="6.7109375" style="4"/>
+    <col min="11" max="11" width="6.7109375" style="15"/>
+    <col min="12" max="12" width="6.7109375" style="4"/>
+    <col min="13" max="13" width="6.7109375" style="15"/>
+    <col min="14" max="14" width="6.7109375" style="4"/>
+    <col min="15" max="15" width="6.7109375" style="15"/>
+    <col min="16" max="16" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.7109375" style="15"/>
+    <col min="18" max="18" width="6.7109375" style="26"/>
+    <col min="19" max="22" width="6.7109375" style="4"/>
+    <col min="23" max="23" width="30.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="6.7109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="102" t="s">
+    <row r="1" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="102"/>
-      <c r="H1" s="102"/>
-      <c r="I1" s="102"/>
-      <c r="J1" s="102"/>
-      <c r="K1" s="102"/>
-      <c r="L1" s="102"/>
-      <c r="M1" s="102"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
@@ -5863,19 +5863,19 @@
       <c r="R1" s="3"/>
       <c r="S1" s="3"/>
     </row>
-    <row r="2" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="96" t="s">
+    <row r="2" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="97"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="79"/>
       <c r="I2" s="5">
         <f>'two way slab design'!D10/'two way slab design'!D11</f>
-        <v>1.3255515883914677</v>
+        <v>1.1304252145634153</v>
       </c>
       <c r="K2" s="4"/>
       <c r="M2" s="4"/>
@@ -5883,40 +5883,40 @@
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
     </row>
-    <row r="3" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="96" t="s">
+    <row r="3" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
-      <c r="H3" s="97"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="79"/>
       <c r="I3" s="5">
         <f>P3</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K3" s="4"/>
       <c r="M3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4">
         <f>IF('two way slab design'!T21=W5,B5,IF('two way slab design'!T21=W6,B6,IF('two way slab design'!T21=W7,B7,IF('two way slab design'!T21=W8,B8,IF('two way slab design'!T21=W9,B9,IF('two way slab design'!T21=W10,B10,IF('two way slab design'!T21=W11,B11,IF('two way slab design'!T21=W12,B12,IF('two way slab design'!T21=W13,B13,"ERROR")))))))))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="104"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="104"/>
-      <c r="H4" s="104"/>
+      <c r="C4" s="80"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="80"/>
       <c r="I4" s="4"/>
       <c r="K4" s="4"/>
       <c r="M4" s="4"/>
@@ -5924,18 +5924,18 @@
       <c r="Q4" s="4"/>
       <c r="R4" s="6"/>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B5" s="8">
         <v>1</v>
       </c>
-      <c r="C5" s="90" t="s">
+      <c r="C5" s="75" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="75"/>
+      <c r="F5" s="75"/>
+      <c r="G5" s="75"/>
+      <c r="H5" s="75"/>
       <c r="I5" s="4"/>
       <c r="K5" s="4"/>
       <c r="M5" s="4"/>
@@ -5951,18 +5951,18 @@
       <c r="AA5" s="31"/>
       <c r="AB5" s="31"/>
     </row>
-    <row r="6" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8">
         <v>2</v>
       </c>
-      <c r="C6" s="90" t="s">
+      <c r="C6" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="90"/>
-      <c r="E6" s="90"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
+      <c r="D6" s="75"/>
+      <c r="E6" s="75"/>
+      <c r="F6" s="75"/>
+      <c r="G6" s="75"/>
+      <c r="H6" s="75"/>
       <c r="I6" s="4"/>
       <c r="K6" s="4"/>
       <c r="M6" s="4"/>
@@ -5978,21 +5978,21 @@
       <c r="AA6" s="31"/>
       <c r="AB6" s="31"/>
     </row>
-    <row r="7" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8">
         <v>3</v>
       </c>
-      <c r="C7" s="90" t="s">
+      <c r="C7" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="90"/>
-      <c r="E7" s="90"/>
-      <c r="F7" s="90"/>
-      <c r="G7" s="90"/>
-      <c r="H7" s="90"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="75"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="96"/>
-      <c r="K7" s="97"/>
+      <c r="J7" s="77"/>
+      <c r="K7" s="79"/>
       <c r="L7" s="9" t="s">
         <v>29</v>
       </c>
@@ -6011,30 +6011,30 @@
       <c r="AA7" s="31"/>
       <c r="AB7" s="31"/>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B8" s="8">
         <v>4</v>
       </c>
-      <c r="C8" s="90" t="s">
+      <c r="C8" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="90"/>
-      <c r="E8" s="90"/>
-      <c r="F8" s="90"/>
-      <c r="G8" s="90"/>
-      <c r="H8" s="90"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
+      <c r="G8" s="75"/>
+      <c r="H8" s="75"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="98" t="s">
+      <c r="J8" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="99"/>
+      <c r="K8" s="82"/>
       <c r="L8" s="11">
         <f>IF($I$3=$A$17,R17,IF($I$3=$A$20,R20,IF($I$3=$A$23,R23,IF($I$3=$A$26,R26,IF($I$3=$A$29,R29,IF($I$3=$A$32,R32,IF($I$3=$A$35,R35,IF($I$3=$A$38,R38,IF($I$3=$A$41,R41,0)))))))))</f>
-        <v>5.2022063535658705E-2</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="M8" s="12">
         <f>IF($I$3=$A$17,S17,IF($I$3=$A$20,S20,IF($I$3=$A$23,S23,IF($I$3=$A$26,S26,IF($I$3=$A$29,S29,IF($I$3=$A$32,S32,IF($I$3=$A$35,S35,IF($I$3=$A$38,S38,IF($I$3=$A$41,S41,0)))))))))</f>
-        <v>3.6999999999999998E-2</v>
+        <v>4.7E-2</v>
       </c>
       <c r="O8" s="4"/>
       <c r="Q8" s="4"/>
@@ -6048,30 +6048,30 @@
       <c r="AA8" s="31"/>
       <c r="AB8" s="31"/>
     </row>
-    <row r="9" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8">
         <v>5</v>
       </c>
-      <c r="C9" s="90" t="s">
+      <c r="C9" s="75" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="90"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="90"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="75"/>
+      <c r="H9" s="75"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="100" t="s">
+      <c r="J9" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="101"/>
+      <c r="K9" s="84"/>
       <c r="L9" s="13">
         <f>IF($I$3=$A$17,R18,IF($I$3=$A$20,R21,IF($I$3=$A$23,R24,IF($I$3=$A$26,R27,IF($I$3=$A$29,R30,IF($I$3=$A$32,R33,IF($I$3=$A$35,R36,IF($I$3=$A$38,R39,IF($I$3=$A$41,R42,0)))))))))</f>
-        <v>3.9511031767829351E-2</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="M9" s="14">
         <f>IF($I$3=$A$17,S18,IF($I$3=$A$20,S21,IF($I$3=$A$23,S24,IF($I$3=$A$26,S27,IF($I$3=$A$29,S30,IF($I$3=$A$32,S33,IF($I$3=$A$35,S36,IF($I$3=$A$38,S39,IF($I$3=$A$41,S42,0)))))))))</f>
-        <v>2.8000000000000001E-2</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="O9" s="4"/>
       <c r="Q9" s="4"/>
@@ -6085,18 +6085,18 @@
       <c r="AA9" s="31"/>
       <c r="AB9" s="31"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B10" s="8">
         <v>6</v>
       </c>
-      <c r="C10" s="90" t="s">
+      <c r="C10" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="90"/>
-      <c r="E10" s="90"/>
-      <c r="F10" s="90"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="90"/>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="75"/>
       <c r="I10" s="4"/>
       <c r="K10" s="4"/>
       <c r="M10" s="4"/>
@@ -6112,18 +6112,18 @@
       <c r="AA10" s="31"/>
       <c r="AB10" s="31"/>
     </row>
-    <row r="11" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="8">
         <v>7</v>
       </c>
-      <c r="C11" s="91" t="s">
+      <c r="C11" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="91"/>
-      <c r="E11" s="91"/>
-      <c r="F11" s="91"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="91"/>
+      <c r="D11" s="87"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="87"/>
+      <c r="G11" s="87"/>
+      <c r="H11" s="87"/>
       <c r="I11" s="4"/>
       <c r="K11" s="4"/>
       <c r="M11" s="4"/>
@@ -6139,18 +6139,18 @@
       <c r="AA11" s="32"/>
       <c r="AB11" s="32"/>
     </row>
-    <row r="12" spans="1:28" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="8">
         <v>8</v>
       </c>
-      <c r="C12" s="91" t="s">
+      <c r="C12" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="91"/>
-      <c r="E12" s="91"/>
-      <c r="F12" s="91"/>
-      <c r="G12" s="91"/>
-      <c r="H12" s="91"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="87"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
       <c r="I12" s="4"/>
       <c r="K12" s="4"/>
       <c r="M12" s="4"/>
@@ -6166,23 +6166,23 @@
       <c r="AA12" s="32"/>
       <c r="AB12" s="32"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B13" s="8">
         <v>9</v>
       </c>
-      <c r="C13" s="90" t="s">
+      <c r="C13" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
+      <c r="D13" s="75"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="75"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="75"/>
       <c r="I13" s="4"/>
       <c r="K13" s="4"/>
       <c r="M13" s="4"/>
       <c r="O13" s="4"/>
-      <c r="R13" s="92" t="s">
+      <c r="R13" s="88" t="s">
         <v>39</v>
       </c>
       <c r="W13" s="31" t="s">
@@ -6194,38 +6194,38 @@
       <c r="AA13" s="31"/>
       <c r="AB13" s="31"/>
     </row>
-    <row r="14" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="R14" s="92"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R14" s="88"/>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
-      <c r="B15" s="93" t="s">
+      <c r="B15" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="93"/>
-      <c r="D15" s="93"/>
-      <c r="E15" s="93"/>
-      <c r="F15" s="93"/>
-      <c r="G15" s="93"/>
-      <c r="H15" s="93"/>
-      <c r="I15" s="93"/>
-      <c r="J15" s="93"/>
-      <c r="K15" s="93"/>
-      <c r="L15" s="93"/>
-      <c r="M15" s="93"/>
-      <c r="N15" s="93"/>
-      <c r="O15" s="93"/>
-      <c r="P15" s="93"/>
-      <c r="Q15" s="93"/>
-      <c r="R15" s="94" t="s">
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+      <c r="K15" s="89"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="89"/>
+      <c r="N15" s="89"/>
+      <c r="O15" s="89"/>
+      <c r="P15" s="89"/>
+      <c r="Q15" s="89"/>
+      <c r="R15" s="90" t="s">
         <v>29</v>
       </c>
-      <c r="S15" s="88" t="s">
+      <c r="S15" s="85" t="s">
         <v>30</v>
       </c>
       <c r="T15" s="2"/>
     </row>
-    <row r="16" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17"/>
       <c r="B16" s="18">
         <v>1</v>
@@ -6239,7 +6239,7 @@
       </c>
       <c r="E16" s="18">
         <f>IF(AND($I$2&gt;=D16,$I$2&lt;=F16),$I$2,0)</f>
-        <v>0</v>
+        <v>1.1304252145634153</v>
       </c>
       <c r="F16" s="18">
         <v>1.2</v>
@@ -6253,7 +6253,7 @@
       </c>
       <c r="I16" s="18">
         <f>IF(AND($I$2&gt;=H16,$I$2&lt;=J16),$I$2,0)</f>
-        <v>1.3255515883914677</v>
+        <v>0</v>
       </c>
       <c r="J16" s="18">
         <v>1.4</v>
@@ -6283,10 +6283,10 @@
         <f>IF(AND($I$2&gt;=P16),$I$2,0)</f>
         <v>0</v>
       </c>
-      <c r="R16" s="95"/>
-      <c r="S16" s="89"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="R16" s="91"/>
+      <c r="S16" s="86"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="17">
         <v>1</v>
       </c>
@@ -6302,7 +6302,7 @@
       </c>
       <c r="E17" s="20">
         <f>IF($E$16&gt;0,(((F17-D17)/($F$16-$D$16))*($E$16-$D$16))+D17,0)</f>
-        <v>0</v>
+        <v>3.882551287380491E-2</v>
       </c>
       <c r="F17" s="19">
         <v>4.2999999999999997E-2</v>
@@ -6316,7 +6316,7 @@
       </c>
       <c r="I17" s="20">
         <f>IF($I$16&gt;0,(((J17-H17)/($J$16-$H$16))*($I$16-$H$16))+H17,0)</f>
-        <v>4.8022063535658709E-2</v>
+        <v>0</v>
       </c>
       <c r="J17" s="19">
         <v>5.0999999999999997E-2</v>
@@ -6348,13 +6348,13 @@
       </c>
       <c r="R17" s="21">
         <f>MAX(C17,E17,G17,I17,K17,M17,O17)</f>
-        <v>4.8022063535658709E-2</v>
+        <v>3.882551287380491E-2</v>
       </c>
       <c r="S17" s="22">
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="17"/>
       <c r="B18" s="19">
         <v>2.4E-2</v>
@@ -6368,7 +6368,7 @@
       </c>
       <c r="E18" s="20">
         <f t="shared" ref="E18:E42" si="1">IF($E$16&gt;0,(((F18-D18)/($F$16-$D$16))*($E$16-$D$16))+D18,0)</f>
-        <v>0</v>
+        <v>2.9217008582536608E-2</v>
       </c>
       <c r="F18" s="19">
         <v>3.2000000000000001E-2</v>
@@ -6382,7 +6382,7 @@
       </c>
       <c r="I18" s="20">
         <f t="shared" ref="I18:I42" si="2">IF($I$16&gt;0,(((J18-H18)/($J$16-$H$16))*($I$16-$H$16))+H18,0)</f>
-        <v>3.676654765174403E-2</v>
+        <v>0</v>
       </c>
       <c r="J18" s="19">
         <v>3.9E-2</v>
@@ -6414,13 +6414,13 @@
       </c>
       <c r="R18" s="21">
         <f t="shared" ref="R18:R42" si="6">MAX(C18,E18,G18,I18,K18,M18,O18)</f>
-        <v>3.676654765174403E-2</v>
+        <v>2.9217008582536608E-2</v>
       </c>
       <c r="S18" s="22">
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="17"/>
       <c r="B19" s="19"/>
       <c r="C19" s="20"/>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="S19" s="22"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="17">
         <v>2</v>
       </c>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="E20" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.452126072817076E-2</v>
       </c>
       <c r="F20" s="19">
         <v>4.8000000000000001E-2</v>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="I20" s="20">
         <f t="shared" si="2"/>
-        <v>5.2022063535658705E-2</v>
+        <v>0</v>
       </c>
       <c r="J20" s="19">
         <v>5.5E-2</v>
@@ -6506,13 +6506,13 @@
       </c>
       <c r="R20" s="21">
         <f t="shared" si="6"/>
-        <v>5.2022063535658705E-2</v>
+        <v>4.452126072817076E-2</v>
       </c>
       <c r="S20" s="22">
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="B21" s="19">
         <v>2.8000000000000001E-2</v>
@@ -6526,7 +6526,7 @@
       </c>
       <c r="E21" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.3217008582536608E-2</v>
       </c>
       <c r="F21" s="19">
         <v>3.5999999999999997E-2</v>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="I21" s="20">
         <f t="shared" si="2"/>
-        <v>3.9511031767829351E-2</v>
+        <v>0</v>
       </c>
       <c r="J21" s="19">
         <v>4.1000000000000002E-2</v>
@@ -6572,13 +6572,13 @@
       </c>
       <c r="R21" s="21">
         <f t="shared" si="6"/>
-        <v>3.9511031767829351E-2</v>
+        <v>3.3217008582536608E-2</v>
       </c>
       <c r="S21" s="22">
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="17"/>
       <c r="B22" s="19"/>
       <c r="C22" s="20"/>
@@ -6602,7 +6602,7 @@
       </c>
       <c r="S22" s="22"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="17">
         <v>3</v>
       </c>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="E23" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.6434017165073213E-2</v>
       </c>
       <c r="F23" s="19">
         <v>5.1999999999999998E-2</v>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="I23" s="20">
         <f t="shared" si="2"/>
-        <v>5.8533095303488061E-2</v>
+        <v>0</v>
       </c>
       <c r="J23" s="19">
         <v>6.3E-2</v>
@@ -6664,13 +6664,13 @@
       </c>
       <c r="R23" s="21">
         <f t="shared" si="6"/>
-        <v>5.8533095303488061E-2</v>
+        <v>4.6434017165073213E-2</v>
       </c>
       <c r="S23" s="22">
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="17"/>
       <c r="B24" s="19">
         <v>2.8000000000000001E-2</v>
@@ -6684,7 +6684,7 @@
       </c>
       <c r="E24" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.4825512873804913E-2</v>
       </c>
       <c r="F24" s="19">
         <v>3.9E-2</v>
@@ -6698,7 +6698,7 @@
       </c>
       <c r="I24" s="20">
         <f t="shared" si="2"/>
-        <v>4.4766547651744031E-2</v>
+        <v>0</v>
       </c>
       <c r="J24" s="19">
         <v>4.7E-2</v>
@@ -6730,13 +6730,13 @@
       </c>
       <c r="R24" s="21">
         <f t="shared" si="6"/>
-        <v>4.4766547651744031E-2</v>
+        <v>3.4825512873804913E-2</v>
       </c>
       <c r="S24" s="22">
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="B25" s="19"/>
       <c r="C25" s="20"/>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="S25" s="22"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="17">
         <v>4</v>
       </c>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="E26" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="F26" s="19">
         <v>0.06</v>
@@ -6790,7 +6790,7 @@
       </c>
       <c r="I26" s="20">
         <f t="shared" si="2"/>
-        <v>6.6533095303488055E-2</v>
+        <v>0</v>
       </c>
       <c r="J26" s="19">
         <v>7.0999999999999994E-2</v>
@@ -6822,13 +6822,13 @@
       </c>
       <c r="R26" s="21">
         <f t="shared" si="6"/>
-        <v>6.6533095303488055E-2</v>
+        <v>5.5129765019439066E-2</v>
       </c>
       <c r="S26" s="22">
         <v>4.7E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
       <c r="B27" s="19">
         <v>3.5000000000000003E-2</v>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="E27" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="F27" s="19">
         <v>4.4999999999999998E-2</v>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="I27" s="20">
         <f t="shared" si="2"/>
-        <v>5.002206353565871E-2</v>
+        <v>0</v>
       </c>
       <c r="J27" s="19">
         <v>5.2999999999999999E-2</v>
@@ -6888,13 +6888,13 @@
       </c>
       <c r="R27" s="21">
         <f t="shared" si="6"/>
-        <v>5.002206353565871E-2</v>
+        <v>4.1521260728170764E-2</v>
       </c>
       <c r="S27" s="22">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="17"/>
       <c r="B28" s="19"/>
       <c r="C28" s="20"/>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="S28" s="22"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="17">
         <v>5</v>
       </c>
@@ -6934,7 +6934,7 @@
       </c>
       <c r="E29" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.9912756436902454E-2</v>
       </c>
       <c r="F29" s="19">
         <v>5.1999999999999998E-2</v>
@@ -6948,7 +6948,7 @@
       </c>
       <c r="I29" s="20">
         <f t="shared" si="2"/>
-        <v>5.6766547651744027E-2</v>
+        <v>0</v>
       </c>
       <c r="J29" s="19">
         <v>5.8999999999999997E-2</v>
@@ -6980,11 +6980,11 @@
       </c>
       <c r="R29" s="21">
         <f t="shared" si="6"/>
-        <v>5.6766547651744027E-2</v>
+        <v>4.9912756436902454E-2</v>
       </c>
       <c r="S29" s="22"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="17"/>
       <c r="B30" s="19">
         <v>3.5000000000000003E-2</v>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="E30" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3.7912756436902458E-2</v>
       </c>
       <c r="F30" s="19">
         <v>0.04</v>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="I30" s="20">
         <f t="shared" si="2"/>
-        <v>4.3255515883914672E-2</v>
+        <v>0</v>
       </c>
       <c r="J30" s="19">
         <v>4.3999999999999997E-2</v>
@@ -7044,13 +7044,13 @@
       </c>
       <c r="R30" s="21">
         <f t="shared" si="6"/>
-        <v>4.3255515883914672E-2</v>
+        <v>3.7912756436902458E-2</v>
       </c>
       <c r="S30" s="22">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
       <c r="B31" s="19"/>
       <c r="C31" s="20"/>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="S31" s="22"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="17">
         <v>6</v>
       </c>
@@ -7126,7 +7126,7 @@
         <v>4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="17"/>
       <c r="B33" s="19">
         <v>3.5000000000000003E-2</v>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="E33" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.5434017165073212E-2</v>
       </c>
       <c r="F33" s="19">
         <v>5.0999999999999997E-2</v>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="I33" s="20">
         <f t="shared" si="2"/>
-        <v>5.8533095303488061E-2</v>
+        <v>0</v>
       </c>
       <c r="J33" s="19">
         <v>6.3E-2</v>
@@ -7186,13 +7186,13 @@
       </c>
       <c r="R33" s="21">
         <f t="shared" si="6"/>
-        <v>5.8533095303488061E-2</v>
+        <v>4.5434017165073212E-2</v>
       </c>
       <c r="S33" s="22">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
       <c r="B34" s="19"/>
       <c r="C34" s="20"/>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="S34" s="22"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="17">
         <v>7</v>
       </c>
@@ -7232,7 +7232,7 @@
       </c>
       <c r="E35" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6.6129765019439068E-2</v>
       </c>
       <c r="F35" s="19">
         <v>7.0999999999999994E-2</v>
@@ -7246,7 +7246,7 @@
       </c>
       <c r="I35" s="20">
         <f t="shared" si="2"/>
-        <v>7.70220635356587E-2</v>
+        <v>0</v>
       </c>
       <c r="J35" s="19">
         <v>0.08</v>
@@ -7278,11 +7278,11 @@
       </c>
       <c r="R35" s="21">
         <f t="shared" si="6"/>
-        <v>7.70220635356587E-2</v>
+        <v>6.6129765019439068E-2</v>
       </c>
       <c r="S35" s="22"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="17"/>
       <c r="B36" s="19">
         <v>4.2999999999999997E-2</v>
@@ -7296,7 +7296,7 @@
       </c>
       <c r="E36" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4.9521260728170764E-2</v>
       </c>
       <c r="F36" s="19">
         <v>5.2999999999999999E-2</v>
@@ -7310,7 +7310,7 @@
       </c>
       <c r="I36" s="20">
         <f t="shared" si="2"/>
-        <v>5.7766547651744028E-2</v>
+        <v>0</v>
       </c>
       <c r="J36" s="19">
         <v>0.06</v>
@@ -7342,13 +7342,13 @@
       </c>
       <c r="R36" s="21">
         <f t="shared" si="6"/>
-        <v>5.7766547651744028E-2</v>
+        <v>4.9521260728170764E-2</v>
       </c>
       <c r="S36" s="22">
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="17"/>
       <c r="B37" s="19"/>
       <c r="C37" s="20"/>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="S37" s="22"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="17">
         <v>8</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>5.7000000000000002E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="17"/>
       <c r="B39" s="19">
         <v>4.2999999999999997E-2</v>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="E39" s="20">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5.3434017165073212E-2</v>
       </c>
       <c r="F39" s="19">
         <v>5.8999999999999997E-2</v>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="I39" s="20">
         <f t="shared" si="2"/>
-        <v>6.6533095303488055E-2</v>
+        <v>0</v>
       </c>
       <c r="J39" s="19">
         <v>7.0999999999999994E-2</v>
@@ -7484,13 +7484,13 @@
       </c>
       <c r="R39" s="21">
         <f t="shared" si="6"/>
-        <v>6.6533095303488055E-2</v>
+        <v>5.3434017165073212E-2</v>
       </c>
       <c r="S39" s="22">
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="17"/>
       <c r="B40" s="19"/>
       <c r="C40" s="20"/>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="S40" s="22"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="17">
         <v>9</v>
       </c>
@@ -7564,7 +7564,7 @@
       </c>
       <c r="S41" s="22"/>
     </row>
-    <row r="42" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="23"/>
       <c r="B42" s="24">
         <v>5.6000000000000001E-2</v>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="E42" s="25">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6.0868034330146432E-2</v>
       </c>
       <c r="F42" s="24">
         <v>7.1999999999999995E-2</v>
@@ -7592,7 +7592,7 @@
       </c>
       <c r="I42" s="25">
         <f t="shared" si="2"/>
-        <v>8.0533095303488067E-2</v>
+        <v>0</v>
       </c>
       <c r="J42" s="24">
         <v>8.5000000000000006E-2</v>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="R42" s="21">
         <f t="shared" si="6"/>
-        <v>8.0533095303488067E-2</v>
+        <v>6.0868034330146432E-2</v>
       </c>
       <c r="S42" s="14">
         <v>5.6000000000000001E-2</v>
@@ -7632,18 +7632,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="J9:K9"/>
     <mergeCell ref="S15:S16"/>
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="C11:H11"/>
@@ -7652,6 +7640,18 @@
     <mergeCell ref="R13:R14"/>
     <mergeCell ref="B15:Q15"/>
     <mergeCell ref="R15:R16"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="C5:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7660,17 +7660,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>48</v>
       </c>
@@ -7679,7 +7679,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>47</v>
       </c>
@@ -7688,7 +7688,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>46</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>53</v>
       </c>
@@ -7705,7 +7705,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>42</v>
       </c>
@@ -7731,10 +7731,10 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7">
         <f>'two way slab design'!C36</f>
-        <v>6.5986603309068741</v>
+        <v>10.892081088866247</v>
       </c>
       <c r="F7">
         <f>0.416*0.87*0.87*$D$4*$D$4/(0.362*$D$3*$D$5)</f>
@@ -7746,29 +7746,29 @@
       </c>
       <c r="H7">
         <f>B7*10^6</f>
-        <v>6598660.3309068745</v>
+        <v>10892081.088866247</v>
       </c>
       <c r="I7">
         <f>G7*G7-4*F7*H7</f>
-        <v>1799227335.2407763</v>
+        <v>1612504806.038156</v>
       </c>
       <c r="J7">
         <f>IF(I7&gt;0,((-G7+SQRT(I7))/(2*F7)),"cant solve")</f>
-        <v>4051.1159617063336</v>
+        <v>3947.125435564566</v>
       </c>
       <c r="K7">
         <f>IF(I7&gt;0,((-G7-SQRT(I7))/(2*F7)),"cant solve")</f>
-        <v>149.81242025653103</v>
+        <v>253.80294639829856</v>
       </c>
       <c r="L7">
         <f>IF(J7&gt;K7,K7,J7)</f>
-        <v>149.81242025653103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>253.80294639829856</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8">
         <f>'two way slab design'!D36</f>
-        <v>5.011717341448124</v>
+        <v>8.2034258372718725</v>
       </c>
       <c r="F8">
         <f t="shared" ref="F8:F10" si="0">0.416*0.87*0.87*$D$4*$D$4/(0.362*$D$3*$D$5)</f>
@@ -7780,29 +7780,29 @@
       </c>
       <c r="H8">
         <f t="shared" ref="H8:H10" si="2">B8*10^6</f>
-        <v>5011717.3414481236</v>
+        <v>8203425.8372718729</v>
       </c>
       <c r="I8">
         <f t="shared" ref="I8:I10" si="3">G8*G8-4*F8*H8</f>
-        <v>1868244099.5871952</v>
+        <v>1729435462.7414186</v>
       </c>
       <c r="J8">
         <f t="shared" ref="J8:J10" si="4">IF(I8&gt;0,((-G8+SQRT(I8))/(2*F8)),"cant solve")</f>
-        <v>4088.1765390561109</v>
+        <v>4012.9089792535533</v>
       </c>
       <c r="K8">
         <f t="shared" ref="K8:K10" si="5">IF(I8&gt;0,((-G8-SQRT(I8))/(2*F8)),"cant solve")</f>
-        <v>112.75184290675337</v>
+        <v>188.01940270931087</v>
       </c>
       <c r="L8">
         <f t="shared" ref="L8:L10" si="6">IF(J8&gt;K8,K8,J8)</f>
-        <v>112.75184290675337</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>188.01940270931087</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9">
         <f>'two way slab design'!E36</f>
-        <v>4.6932092971706236</v>
+        <v>9.2858696385918762</v>
       </c>
       <c r="F9">
         <f t="shared" si="0"/>
@@ -7814,29 +7814,29 @@
       </c>
       <c r="H9">
         <f t="shared" si="2"/>
-        <v>4693209.2971706232</v>
+        <v>9285869.6385918763</v>
       </c>
       <c r="I9">
         <f t="shared" si="3"/>
-        <v>1882096137.6127303</v>
+        <v>1682359563.1973372</v>
       </c>
       <c r="J9">
         <f t="shared" si="4"/>
-        <v>4095.5318461380639</v>
+        <v>3986.7006566552895</v>
       </c>
       <c r="K9">
         <f t="shared" si="5"/>
-        <v>105.39653582479998</v>
+        <v>214.22772530757535</v>
       </c>
       <c r="L9">
         <f t="shared" si="6"/>
-        <v>105.39653582479998</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>214.22772530757535</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10">
         <f>'two way slab design'!F36</f>
-        <v>3.551617846507499</v>
+        <v>6.9150093053343742</v>
       </c>
       <c r="F10">
         <f t="shared" si="0"/>
@@ -7848,23 +7848,23 @@
       </c>
       <c r="H10">
         <f t="shared" si="2"/>
-        <v>3551617.846507499</v>
+        <v>6915009.3053343743</v>
       </c>
       <c r="I10">
         <f t="shared" si="3"/>
-        <v>1931744391.3015256</v>
+        <v>1785469195.9980171</v>
       </c>
       <c r="J10">
         <f t="shared" si="4"/>
-        <v>4121.6747388798049</v>
+        <v>4043.6436319266199</v>
       </c>
       <c r="K10">
         <f t="shared" si="5"/>
-        <v>79.253643083059629</v>
+        <v>157.28475003624399</v>
       </c>
       <c r="L10">
         <f t="shared" si="6"/>
-        <v>79.253643083059629</v>
+        <v>157.28475003624399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>